<commit_message>
effect size meadian and iqt
</commit_message>
<xml_diff>
--- a/02.FOMD/02.metadata_structure/10_FOMD_metadata_synthesis_short.xlsx
+++ b/02.FOMD/02.metadata_structure/10_FOMD_metadata_synthesis_short.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="3044" documentId="14_{431D3801-6596-4146-883F-336ABD7CEFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE7C217D-E428-40D6-8FB6-826D5C0759D2}"/>
   <bookViews>
-    <workbookView xWindow="-57710" yWindow="-110" windowWidth="29020" windowHeight="15700" xr2:uid="{FAB1A633-BA4D-4813-8605-DC3F4755D7C7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{FAB1A633-BA4D-4813-8605-DC3F4755D7C7}"/>
   </bookViews>
   <sheets>
     <sheet name="10_FOMD_metadata_synthesis" sheetId="1" r:id="rId1"/>
@@ -33072,6 +33072,24 @@
   </sheetData>
   <autoFilter ref="A1:S321" xr:uid="{82619C4B-D6B1-486E-87C6-D2252668E253}"/>
   <mergeCells count="27">
+    <mergeCell ref="O544:O545"/>
+    <mergeCell ref="P544:P545"/>
+    <mergeCell ref="Q544:Q545"/>
+    <mergeCell ref="O548:O549"/>
+    <mergeCell ref="P548:P549"/>
+    <mergeCell ref="Q548:Q549"/>
+    <mergeCell ref="O558:O559"/>
+    <mergeCell ref="P558:P559"/>
+    <mergeCell ref="Q558:Q559"/>
+    <mergeCell ref="O560:O561"/>
+    <mergeCell ref="P560:P561"/>
+    <mergeCell ref="Q560:Q561"/>
+    <mergeCell ref="O566:O568"/>
+    <mergeCell ref="P566:P568"/>
+    <mergeCell ref="Q566:Q568"/>
+    <mergeCell ref="O569:O571"/>
+    <mergeCell ref="P569:P571"/>
+    <mergeCell ref="Q569:Q571"/>
     <mergeCell ref="O556:O557"/>
     <mergeCell ref="P556:P557"/>
     <mergeCell ref="Q556:Q557"/>
@@ -33081,24 +33099,6 @@
     <mergeCell ref="P554:P555"/>
     <mergeCell ref="Q554:Q555"/>
     <mergeCell ref="O550:O551"/>
-    <mergeCell ref="O566:O568"/>
-    <mergeCell ref="P566:P568"/>
-    <mergeCell ref="Q566:Q568"/>
-    <mergeCell ref="O569:O571"/>
-    <mergeCell ref="P569:P571"/>
-    <mergeCell ref="Q569:Q571"/>
-    <mergeCell ref="O558:O559"/>
-    <mergeCell ref="P558:P559"/>
-    <mergeCell ref="Q558:Q559"/>
-    <mergeCell ref="O560:O561"/>
-    <mergeCell ref="P560:P561"/>
-    <mergeCell ref="Q560:Q561"/>
-    <mergeCell ref="O544:O545"/>
-    <mergeCell ref="P544:P545"/>
-    <mergeCell ref="Q544:Q545"/>
-    <mergeCell ref="O548:O549"/>
-    <mergeCell ref="P548:P549"/>
-    <mergeCell ref="Q548:Q549"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="Q7" r:id="rId1" display="Abbreviation of the journal name. We use WoS abbreviations that can be found here: https://images.webofknowledge.com/images/help/WOS/A_abrvjt.html" xr:uid="{B4DADD6B-F846-45B3-933B-5F25CC9FEF24}"/>
@@ -43675,24 +43675,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="D553:D554"/>
-    <mergeCell ref="E553:E554"/>
-    <mergeCell ref="F553:F554"/>
-    <mergeCell ref="D557:D558"/>
-    <mergeCell ref="E557:E558"/>
-    <mergeCell ref="F557:F558"/>
-    <mergeCell ref="D559:D560"/>
-    <mergeCell ref="E559:E560"/>
-    <mergeCell ref="F559:F560"/>
-    <mergeCell ref="D563:D564"/>
-    <mergeCell ref="E563:E564"/>
-    <mergeCell ref="F563:F564"/>
-    <mergeCell ref="D565:D566"/>
-    <mergeCell ref="E565:E566"/>
-    <mergeCell ref="F565:F566"/>
-    <mergeCell ref="D567:D568"/>
-    <mergeCell ref="E567:E568"/>
-    <mergeCell ref="F567:F568"/>
     <mergeCell ref="D578:D580"/>
     <mergeCell ref="E578:E580"/>
     <mergeCell ref="F578:F580"/>
@@ -43702,6 +43684,24 @@
     <mergeCell ref="D575:D577"/>
     <mergeCell ref="E575:E577"/>
     <mergeCell ref="F575:F577"/>
+    <mergeCell ref="D565:D566"/>
+    <mergeCell ref="E565:E566"/>
+    <mergeCell ref="F565:F566"/>
+    <mergeCell ref="D567:D568"/>
+    <mergeCell ref="E567:E568"/>
+    <mergeCell ref="F567:F568"/>
+    <mergeCell ref="D559:D560"/>
+    <mergeCell ref="E559:E560"/>
+    <mergeCell ref="F559:F560"/>
+    <mergeCell ref="D563:D564"/>
+    <mergeCell ref="E563:E564"/>
+    <mergeCell ref="F563:F564"/>
+    <mergeCell ref="D553:D554"/>
+    <mergeCell ref="E553:E554"/>
+    <mergeCell ref="F553:F554"/>
+    <mergeCell ref="D557:D558"/>
+    <mergeCell ref="E557:E558"/>
+    <mergeCell ref="F557:F558"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F7" r:id="rId1" display="Abbreviation of the journal name. We use WoS abbreviations that can be found here: https://images.webofknowledge.com/images/help/WOS/A_abrvjt.html" xr:uid="{6BB52E4D-01E2-44A6-B6CC-352383FA2940}"/>
@@ -43713,6 +43713,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4b26243c-b736-4d9c-b036-479be2ad88a1">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="432dd258-9dce-4cb3-b611-c68c0fbce7f3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005BE3C66ACF4393458051577D36AC6C25" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4e0e0d96de7fb32b1678b66c28514d8e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4b26243c-b736-4d9c-b036-479be2ad88a1" xmlns:ns3="432dd258-9dce-4cb3-b611-c68c0fbce7f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac451aab8c96dec805c937cbafca7133" ns2:_="" ns3:_="">
     <xsd:import namespace="4b26243c-b736-4d9c-b036-479be2ad88a1"/>
@@ -43913,27 +43933,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63F80AE0-5CF8-441A-8E3E-6D76A3390D5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4b26243c-b736-4d9c-b036-479be2ad88a1"/>
+    <ds:schemaRef ds:uri="432dd258-9dce-4cb3-b611-c68c0fbce7f3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4b26243c-b736-4d9c-b036-479be2ad88a1">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="432dd258-9dce-4cb3-b611-c68c0fbce7f3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0C90B0A-DBBE-4147-B2EE-79946A8DC171}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC19592A-9F30-4B32-9428-1D9634B8A0D4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -43950,23 +43969,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0C90B0A-DBBE-4147-B2EE-79946A8DC171}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63F80AE0-5CF8-441A-8E3E-6D76A3390D5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4b26243c-b736-4d9c-b036-479be2ad88a1"/>
-    <ds:schemaRef ds:uri="432dd258-9dce-4cb3-b611-c68c0fbce7f3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fixing errors in datasets
</commit_message>
<xml_diff>
--- a/02.FOMD/02.metadata_structure/10_FOMD_metadata_synthesis_short.xlsx
+++ b/02.FOMD/02.metadata_structure/10_FOMD_metadata_synthesis_short.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar.sharepoint.com/sites/Alliance-AgroecologyKnowledgeHub/Shared Documents/General/Agroecology_Evidence_Hub/02.FOMD/02.metadata_structure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3050" documentId="14_{431D3801-6596-4146-883F-336ABD7CEFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{178109FE-65A5-42B3-8323-F656C62B27EA}"/>
+  <xr:revisionPtr revIDLastSave="3057" documentId="14_{431D3801-6596-4146-883F-336ABD7CEFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28C25BDE-0F87-423D-B6C7-5ED6DE029526}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{FAB1A633-BA4D-4813-8605-DC3F4755D7C7}"/>
+    <workbookView xWindow="-57710" yWindow="-110" windowWidth="29020" windowHeight="15700" activeTab="2" xr2:uid="{FAB1A633-BA4D-4813-8605-DC3F4755D7C7}"/>
   </bookViews>
   <sheets>
     <sheet name="10_FOMD_metadata_synthesis" sheetId="1" r:id="rId1"/>
@@ -12375,12 +12375,12 @@
     <xf numFmtId="0" fontId="31" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="26" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="63" fillId="63" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -31677,7 +31677,7 @@
       <c r="L544" s="12"/>
       <c r="M544" s="12"/>
       <c r="N544" s="12"/>
-      <c r="O544" s="159" t="s">
+      <c r="O544" s="156" t="s">
         <v>35</v>
       </c>
       <c r="P544" s="157" t="s">
@@ -31705,7 +31705,7 @@
       <c r="L545" s="12"/>
       <c r="M545" s="12"/>
       <c r="N545" s="12"/>
-      <c r="O545" s="159"/>
+      <c r="O545" s="156"/>
       <c r="P545" s="157"/>
       <c r="Q545" s="158"/>
       <c r="R545" s="3" t="s">
@@ -31755,7 +31755,7 @@
       <c r="L548" s="1"/>
       <c r="M548" s="1"/>
       <c r="N548" s="1"/>
-      <c r="O548" s="156" t="s">
+      <c r="O548" s="159" t="s">
         <v>42</v>
       </c>
       <c r="P548" s="157" t="s">
@@ -31783,7 +31783,7 @@
       <c r="L549" s="1"/>
       <c r="M549" s="1"/>
       <c r="N549" s="1"/>
-      <c r="O549" s="156"/>
+      <c r="O549" s="159"/>
       <c r="P549" s="157"/>
       <c r="Q549" s="158"/>
       <c r="R549" s="3" t="s">
@@ -31805,7 +31805,7 @@
       <c r="L550" s="12"/>
       <c r="M550" s="12"/>
       <c r="N550" s="12"/>
-      <c r="O550" s="159" t="s">
+      <c r="O550" s="156" t="s">
         <v>45</v>
       </c>
       <c r="P550" s="157" t="s">
@@ -31833,7 +31833,7 @@
       <c r="L551" s="12"/>
       <c r="M551" s="12"/>
       <c r="N551" s="12"/>
-      <c r="O551" s="159"/>
+      <c r="O551" s="156"/>
       <c r="P551" s="157"/>
       <c r="Q551" s="158"/>
       <c r="R551" s="3" t="s">
@@ -31883,7 +31883,7 @@
       <c r="L554" s="1"/>
       <c r="M554" s="1"/>
       <c r="N554" s="1"/>
-      <c r="O554" s="156" t="s">
+      <c r="O554" s="159" t="s">
         <v>52</v>
       </c>
       <c r="P554" s="157" t="s">
@@ -31911,7 +31911,7 @@
       <c r="L555" s="1"/>
       <c r="M555" s="1"/>
       <c r="N555" s="1"/>
-      <c r="O555" s="156"/>
+      <c r="O555" s="159"/>
       <c r="P555" s="157"/>
       <c r="Q555" s="158"/>
       <c r="R555" s="3" t="s">
@@ -31933,7 +31933,7 @@
       <c r="L556" s="1"/>
       <c r="M556" s="1"/>
       <c r="N556" s="1"/>
-      <c r="O556" s="159" t="s">
+      <c r="O556" s="156" t="s">
         <v>54</v>
       </c>
       <c r="P556" s="157" t="s">
@@ -31961,7 +31961,7 @@
       <c r="L557" s="1"/>
       <c r="M557" s="1"/>
       <c r="N557" s="1"/>
-      <c r="O557" s="159"/>
+      <c r="O557" s="156"/>
       <c r="P557" s="157"/>
       <c r="Q557" s="158"/>
       <c r="R557" s="3" t="s">
@@ -31983,7 +31983,7 @@
       <c r="L558" s="1"/>
       <c r="M558" s="1"/>
       <c r="N558" s="1"/>
-      <c r="O558" s="159" t="s">
+      <c r="O558" s="156" t="s">
         <v>58</v>
       </c>
       <c r="P558" s="157" t="s">
@@ -32011,7 +32011,7 @@
       <c r="L559" s="1"/>
       <c r="M559" s="1"/>
       <c r="N559" s="1"/>
-      <c r="O559" s="159"/>
+      <c r="O559" s="156"/>
       <c r="P559" s="157"/>
       <c r="Q559" s="158"/>
       <c r="R559" s="3" t="s">
@@ -32033,7 +32033,7 @@
       <c r="L560" s="1"/>
       <c r="M560" s="1"/>
       <c r="N560" s="1"/>
-      <c r="O560" s="159" t="s">
+      <c r="O560" s="156" t="s">
         <v>62</v>
       </c>
       <c r="P560" s="157" t="s">
@@ -32061,7 +32061,7 @@
       <c r="L561" s="1"/>
       <c r="M561" s="1"/>
       <c r="N561" s="1"/>
-      <c r="O561" s="159"/>
+      <c r="O561" s="156"/>
       <c r="P561" s="157"/>
       <c r="Q561" s="158"/>
       <c r="R561" s="3" t="s">
@@ -32193,7 +32193,7 @@
       <c r="L566" s="1"/>
       <c r="M566" s="1"/>
       <c r="N566" s="1"/>
-      <c r="O566" s="156" t="s">
+      <c r="O566" s="159" t="s">
         <v>86</v>
       </c>
       <c r="P566" s="157" t="s">
@@ -32221,7 +32221,7 @@
       <c r="L567" s="1"/>
       <c r="M567" s="1"/>
       <c r="N567" s="1"/>
-      <c r="O567" s="156"/>
+      <c r="O567" s="159"/>
       <c r="P567" s="157"/>
       <c r="Q567" s="158"/>
       <c r="R567" s="3" t="s">
@@ -32243,7 +32243,7 @@
       <c r="L568" s="1"/>
       <c r="M568" s="1"/>
       <c r="N568" s="1"/>
-      <c r="O568" s="156"/>
+      <c r="O568" s="159"/>
       <c r="P568" s="157"/>
       <c r="Q568" s="158"/>
       <c r="R568" s="3" t="s">
@@ -32265,7 +32265,7 @@
       <c r="L569" s="1"/>
       <c r="M569" s="1"/>
       <c r="N569" s="1"/>
-      <c r="O569" s="156" t="s">
+      <c r="O569" s="159" t="s">
         <v>91</v>
       </c>
       <c r="P569" s="157" t="s">
@@ -32293,7 +32293,7 @@
       <c r="L570" s="1"/>
       <c r="M570" s="1"/>
       <c r="N570" s="1"/>
-      <c r="O570" s="156"/>
+      <c r="O570" s="159"/>
       <c r="P570" s="157"/>
       <c r="Q570" s="158"/>
       <c r="R570" s="3" t="s">
@@ -32315,7 +32315,7 @@
       <c r="L571" s="1"/>
       <c r="M571" s="1"/>
       <c r="N571" s="1"/>
-      <c r="O571" s="156"/>
+      <c r="O571" s="159"/>
       <c r="P571" s="157"/>
       <c r="Q571" s="158"/>
       <c r="R571" s="3" t="s">
@@ -33084,6 +33084,24 @@
   </sheetData>
   <autoFilter ref="A1:S321" xr:uid="{82619C4B-D6B1-486E-87C6-D2252668E253}"/>
   <mergeCells count="27">
+    <mergeCell ref="O544:O545"/>
+    <mergeCell ref="P544:P545"/>
+    <mergeCell ref="Q544:Q545"/>
+    <mergeCell ref="O548:O549"/>
+    <mergeCell ref="P548:P549"/>
+    <mergeCell ref="Q548:Q549"/>
+    <mergeCell ref="O558:O559"/>
+    <mergeCell ref="P558:P559"/>
+    <mergeCell ref="Q558:Q559"/>
+    <mergeCell ref="O560:O561"/>
+    <mergeCell ref="P560:P561"/>
+    <mergeCell ref="Q560:Q561"/>
+    <mergeCell ref="O566:O568"/>
+    <mergeCell ref="P566:P568"/>
+    <mergeCell ref="Q566:Q568"/>
+    <mergeCell ref="O569:O571"/>
+    <mergeCell ref="P569:P571"/>
+    <mergeCell ref="Q569:Q571"/>
     <mergeCell ref="O556:O557"/>
     <mergeCell ref="P556:P557"/>
     <mergeCell ref="Q556:Q557"/>
@@ -33093,24 +33111,6 @@
     <mergeCell ref="P554:P555"/>
     <mergeCell ref="Q554:Q555"/>
     <mergeCell ref="O550:O551"/>
-    <mergeCell ref="O566:O568"/>
-    <mergeCell ref="P566:P568"/>
-    <mergeCell ref="Q566:Q568"/>
-    <mergeCell ref="O569:O571"/>
-    <mergeCell ref="P569:P571"/>
-    <mergeCell ref="Q569:Q571"/>
-    <mergeCell ref="O558:O559"/>
-    <mergeCell ref="P558:P559"/>
-    <mergeCell ref="Q558:Q559"/>
-    <mergeCell ref="O560:O561"/>
-    <mergeCell ref="P560:P561"/>
-    <mergeCell ref="Q560:Q561"/>
-    <mergeCell ref="O544:O545"/>
-    <mergeCell ref="P544:P545"/>
-    <mergeCell ref="Q544:Q545"/>
-    <mergeCell ref="O548:O549"/>
-    <mergeCell ref="P548:P549"/>
-    <mergeCell ref="Q548:Q549"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="Q7" r:id="rId1" display="Abbreviation of the journal name. We use WoS abbreviations that can be found here: https://images.webofknowledge.com/images/help/WOS/A_abrvjt.html" xr:uid="{B4DADD6B-F846-45B3-933B-5F25CC9FEF24}"/>
@@ -33368,7 +33368,7 @@
       </c>
       <c r="G11" s="3"/>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" ht="14" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="114" t="s">
         <v>974</v>
@@ -33377,13 +33377,13 @@
         <v>616</v>
       </c>
       <c r="D12" s="115" t="s">
-        <v>1382</v>
+        <v>1383</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F12" s="116" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G12" s="3"/>
     </row>
@@ -33396,13 +33396,13 @@
         <v>616</v>
       </c>
       <c r="D13" s="115" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F13" s="116" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G13" s="3"/>
     </row>
@@ -33567,13 +33567,13 @@
         <v>616</v>
       </c>
       <c r="D22" s="115" t="s">
-        <v>1391</v>
+        <v>1392</v>
       </c>
       <c r="E22" s="92" t="s">
         <v>4</v>
       </c>
       <c r="F22" s="116" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G22" s="92"/>
     </row>
@@ -33586,13 +33586,13 @@
         <v>616</v>
       </c>
       <c r="D23" s="115" t="s">
-        <v>1392</v>
+        <v>1391</v>
       </c>
       <c r="E23" s="92" t="s">
         <v>4</v>
       </c>
       <c r="F23" s="116" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G23" s="92"/>
     </row>
@@ -42897,7 +42897,7 @@
       <c r="A553" s="12"/>
       <c r="B553" s="12"/>
       <c r="C553" s="12"/>
-      <c r="D553" s="159" t="s">
+      <c r="D553" s="156" t="s">
         <v>35</v>
       </c>
       <c r="E553" s="157" t="s">
@@ -42914,7 +42914,7 @@
       <c r="A554" s="12"/>
       <c r="B554" s="12"/>
       <c r="C554" s="12"/>
-      <c r="D554" s="159"/>
+      <c r="D554" s="156"/>
       <c r="E554" s="157"/>
       <c r="F554" s="158"/>
       <c r="G554" s="3" t="s">
@@ -42942,7 +42942,7 @@
       <c r="A557" s="1"/>
       <c r="B557" s="1"/>
       <c r="C557" s="1"/>
-      <c r="D557" s="156" t="s">
+      <c r="D557" s="159" t="s">
         <v>42</v>
       </c>
       <c r="E557" s="157" t="s">
@@ -42959,7 +42959,7 @@
       <c r="A558" s="1"/>
       <c r="B558" s="1"/>
       <c r="C558" s="1"/>
-      <c r="D558" s="156"/>
+      <c r="D558" s="159"/>
       <c r="E558" s="157"/>
       <c r="F558" s="158"/>
       <c r="G558" s="3" t="s">
@@ -42970,7 +42970,7 @@
       <c r="A559" s="12"/>
       <c r="B559" s="12"/>
       <c r="C559" s="12"/>
-      <c r="D559" s="159" t="s">
+      <c r="D559" s="156" t="s">
         <v>45</v>
       </c>
       <c r="E559" s="157" t="s">
@@ -42987,7 +42987,7 @@
       <c r="A560" s="12"/>
       <c r="B560" s="12"/>
       <c r="C560" s="12"/>
-      <c r="D560" s="159"/>
+      <c r="D560" s="156"/>
       <c r="E560" s="157"/>
       <c r="F560" s="158"/>
       <c r="G560" s="3" t="s">
@@ -43015,7 +43015,7 @@
       <c r="A563" s="1"/>
       <c r="B563" s="1"/>
       <c r="C563" s="1"/>
-      <c r="D563" s="156" t="s">
+      <c r="D563" s="159" t="s">
         <v>52</v>
       </c>
       <c r="E563" s="157" t="s">
@@ -43032,7 +43032,7 @@
       <c r="A564" s="1"/>
       <c r="B564" s="1"/>
       <c r="C564" s="1"/>
-      <c r="D564" s="156"/>
+      <c r="D564" s="159"/>
       <c r="E564" s="157"/>
       <c r="F564" s="158"/>
       <c r="G564" s="3" t="s">
@@ -43043,7 +43043,7 @@
       <c r="A565" s="1"/>
       <c r="B565" s="1"/>
       <c r="C565" s="1"/>
-      <c r="D565" s="159" t="s">
+      <c r="D565" s="156" t="s">
         <v>54</v>
       </c>
       <c r="E565" s="157" t="s">
@@ -43060,7 +43060,7 @@
       <c r="A566" s="1"/>
       <c r="B566" s="1"/>
       <c r="C566" s="1"/>
-      <c r="D566" s="159"/>
+      <c r="D566" s="156"/>
       <c r="E566" s="157"/>
       <c r="F566" s="158"/>
       <c r="G566" s="3" t="s">
@@ -43071,7 +43071,7 @@
       <c r="A567" s="1"/>
       <c r="B567" s="1"/>
       <c r="C567" s="1"/>
-      <c r="D567" s="159" t="s">
+      <c r="D567" s="156" t="s">
         <v>58</v>
       </c>
       <c r="E567" s="157" t="s">
@@ -43088,7 +43088,7 @@
       <c r="A568" s="1"/>
       <c r="B568" s="1"/>
       <c r="C568" s="1"/>
-      <c r="D568" s="159"/>
+      <c r="D568" s="156"/>
       <c r="E568" s="157"/>
       <c r="F568" s="158"/>
       <c r="G568" s="3" t="s">
@@ -43099,7 +43099,7 @@
       <c r="A569" s="1"/>
       <c r="B569" s="1"/>
       <c r="C569" s="1"/>
-      <c r="D569" s="159" t="s">
+      <c r="D569" s="156" t="s">
         <v>62</v>
       </c>
       <c r="E569" s="157" t="s">
@@ -43116,7 +43116,7 @@
       <c r="A570" s="1"/>
       <c r="B570" s="1"/>
       <c r="C570" s="1"/>
-      <c r="D570" s="159"/>
+      <c r="D570" s="156"/>
       <c r="E570" s="157"/>
       <c r="F570" s="158"/>
       <c r="G570" s="3" t="s">
@@ -43193,7 +43193,7 @@
       <c r="A575" s="1"/>
       <c r="B575" s="1"/>
       <c r="C575" s="1"/>
-      <c r="D575" s="156" t="s">
+      <c r="D575" s="159" t="s">
         <v>86</v>
       </c>
       <c r="E575" s="157" t="s">
@@ -43210,7 +43210,7 @@
       <c r="A576" s="1"/>
       <c r="B576" s="1"/>
       <c r="C576" s="1"/>
-      <c r="D576" s="156"/>
+      <c r="D576" s="159"/>
       <c r="E576" s="157"/>
       <c r="F576" s="158"/>
       <c r="G576" s="3" t="s">
@@ -43221,7 +43221,7 @@
       <c r="A577" s="1"/>
       <c r="B577" s="1"/>
       <c r="C577" s="1"/>
-      <c r="D577" s="156"/>
+      <c r="D577" s="159"/>
       <c r="E577" s="157"/>
       <c r="F577" s="158"/>
       <c r="G577" s="3" t="s">
@@ -43232,7 +43232,7 @@
       <c r="A578" s="1"/>
       <c r="B578" s="1"/>
       <c r="C578" s="1"/>
-      <c r="D578" s="156" t="s">
+      <c r="D578" s="159" t="s">
         <v>91</v>
       </c>
       <c r="E578" s="157" t="s">
@@ -43249,7 +43249,7 @@
       <c r="A579" s="1"/>
       <c r="B579" s="1"/>
       <c r="C579" s="1"/>
-      <c r="D579" s="156"/>
+      <c r="D579" s="159"/>
       <c r="E579" s="157"/>
       <c r="F579" s="158"/>
       <c r="G579" s="3" t="s">
@@ -43260,7 +43260,7 @@
       <c r="A580" s="1"/>
       <c r="B580" s="1"/>
       <c r="C580" s="1"/>
-      <c r="D580" s="156"/>
+      <c r="D580" s="159"/>
       <c r="E580" s="157"/>
       <c r="F580" s="158"/>
       <c r="G580" s="3" t="s">
@@ -43687,24 +43687,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="D553:D554"/>
-    <mergeCell ref="E553:E554"/>
-    <mergeCell ref="F553:F554"/>
-    <mergeCell ref="D557:D558"/>
-    <mergeCell ref="E557:E558"/>
-    <mergeCell ref="F557:F558"/>
-    <mergeCell ref="D559:D560"/>
-    <mergeCell ref="E559:E560"/>
-    <mergeCell ref="F559:F560"/>
-    <mergeCell ref="D563:D564"/>
-    <mergeCell ref="E563:E564"/>
-    <mergeCell ref="F563:F564"/>
-    <mergeCell ref="D565:D566"/>
-    <mergeCell ref="E565:E566"/>
-    <mergeCell ref="F565:F566"/>
-    <mergeCell ref="D567:D568"/>
-    <mergeCell ref="E567:E568"/>
-    <mergeCell ref="F567:F568"/>
     <mergeCell ref="D578:D580"/>
     <mergeCell ref="E578:E580"/>
     <mergeCell ref="F578:F580"/>
@@ -43714,6 +43696,24 @@
     <mergeCell ref="D575:D577"/>
     <mergeCell ref="E575:E577"/>
     <mergeCell ref="F575:F577"/>
+    <mergeCell ref="D565:D566"/>
+    <mergeCell ref="E565:E566"/>
+    <mergeCell ref="F565:F566"/>
+    <mergeCell ref="D567:D568"/>
+    <mergeCell ref="E567:E568"/>
+    <mergeCell ref="F567:F568"/>
+    <mergeCell ref="D559:D560"/>
+    <mergeCell ref="E559:E560"/>
+    <mergeCell ref="F559:F560"/>
+    <mergeCell ref="D563:D564"/>
+    <mergeCell ref="E563:E564"/>
+    <mergeCell ref="F563:F564"/>
+    <mergeCell ref="D553:D554"/>
+    <mergeCell ref="E553:E554"/>
+    <mergeCell ref="F553:F554"/>
+    <mergeCell ref="D557:D558"/>
+    <mergeCell ref="E557:E558"/>
+    <mergeCell ref="F557:F558"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F7" r:id="rId1" display="Abbreviation of the journal name. We use WoS abbreviations that can be found here: https://images.webofknowledge.com/images/help/WOS/A_abrvjt.html" xr:uid="{6BB52E4D-01E2-44A6-B6CC-352383FA2940}"/>
@@ -43725,6 +43725,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4b26243c-b736-4d9c-b036-479be2ad88a1">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="432dd258-9dce-4cb3-b611-c68c0fbce7f3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005BE3C66ACF4393458051577D36AC6C25" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4e0e0d96de7fb32b1678b66c28514d8e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4b26243c-b736-4d9c-b036-479be2ad88a1" xmlns:ns3="432dd258-9dce-4cb3-b611-c68c0fbce7f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac451aab8c96dec805c937cbafca7133" ns2:_="" ns3:_="">
     <xsd:import namespace="4b26243c-b736-4d9c-b036-479be2ad88a1"/>
@@ -43925,27 +43945,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63F80AE0-5CF8-441A-8E3E-6D76A3390D5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4b26243c-b736-4d9c-b036-479be2ad88a1"/>
+    <ds:schemaRef ds:uri="432dd258-9dce-4cb3-b611-c68c0fbce7f3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4b26243c-b736-4d9c-b036-479be2ad88a1">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="432dd258-9dce-4cb3-b611-c68c0fbce7f3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0C90B0A-DBBE-4147-B2EE-79946A8DC171}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC19592A-9F30-4B32-9428-1D9634B8A0D4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -43962,23 +43981,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0C90B0A-DBBE-4147-B2EE-79946A8DC171}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63F80AE0-5CF8-441A-8E3E-6D76A3390D5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4b26243c-b736-4d9c-b036-479be2ad88a1"/>
-    <ds:schemaRef ds:uri="432dd258-9dce-4cb3-b611-c68c0fbce7f3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
effect size calcualteion ready
</commit_message>
<xml_diff>
--- a/02.FOMD/02.metadata_structure/10_FOMD_metadata_synthesis_short.xlsx
+++ b/02.FOMD/02.metadata_structure/10_FOMD_metadata_synthesis_short.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cgiar.sharepoint.com/sites/Alliance-AgroecologyKnowledgeHub/Shared Documents/General/Agroecology_Evidence_Hub/02.FOMD/02.metadata_structure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3077" documentId="14_{431D3801-6596-4146-883F-336ABD7CEFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E8218A6-A563-4D3D-A425-2A9DFD55F8A1}"/>
+  <xr:revisionPtr revIDLastSave="3078" documentId="14_{431D3801-6596-4146-883F-336ABD7CEFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB51178B-E852-4776-9DF7-67E5D25EF38A}"/>
   <bookViews>
-    <workbookView xWindow="57490" yWindow="-110" windowWidth="29020" windowHeight="15700" activeTab="2" xr2:uid="{FAB1A633-BA4D-4813-8605-DC3F4755D7C7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{FAB1A633-BA4D-4813-8605-DC3F4755D7C7}"/>
   </bookViews>
   <sheets>
     <sheet name="10_FOMD_metadata_synthesis" sheetId="1" r:id="rId1"/>
@@ -12384,12 +12384,12 @@
     <xf numFmtId="0" fontId="31" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="26" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="63" fillId="63" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -31686,7 +31686,7 @@
       <c r="L544" s="12"/>
       <c r="M544" s="12"/>
       <c r="N544" s="12"/>
-      <c r="O544" s="159" t="s">
+      <c r="O544" s="156" t="s">
         <v>35</v>
       </c>
       <c r="P544" s="157" t="s">
@@ -31714,7 +31714,7 @@
       <c r="L545" s="12"/>
       <c r="M545" s="12"/>
       <c r="N545" s="12"/>
-      <c r="O545" s="159"/>
+      <c r="O545" s="156"/>
       <c r="P545" s="157"/>
       <c r="Q545" s="158"/>
       <c r="R545" s="3" t="s">
@@ -31764,7 +31764,7 @@
       <c r="L548" s="1"/>
       <c r="M548" s="1"/>
       <c r="N548" s="1"/>
-      <c r="O548" s="156" t="s">
+      <c r="O548" s="159" t="s">
         <v>42</v>
       </c>
       <c r="P548" s="157" t="s">
@@ -31792,7 +31792,7 @@
       <c r="L549" s="1"/>
       <c r="M549" s="1"/>
       <c r="N549" s="1"/>
-      <c r="O549" s="156"/>
+      <c r="O549" s="159"/>
       <c r="P549" s="157"/>
       <c r="Q549" s="158"/>
       <c r="R549" s="3" t="s">
@@ -31814,7 +31814,7 @@
       <c r="L550" s="12"/>
       <c r="M550" s="12"/>
       <c r="N550" s="12"/>
-      <c r="O550" s="159" t="s">
+      <c r="O550" s="156" t="s">
         <v>45</v>
       </c>
       <c r="P550" s="157" t="s">
@@ -31842,7 +31842,7 @@
       <c r="L551" s="12"/>
       <c r="M551" s="12"/>
       <c r="N551" s="12"/>
-      <c r="O551" s="159"/>
+      <c r="O551" s="156"/>
       <c r="P551" s="157"/>
       <c r="Q551" s="158"/>
       <c r="R551" s="3" t="s">
@@ -31892,7 +31892,7 @@
       <c r="L554" s="1"/>
       <c r="M554" s="1"/>
       <c r="N554" s="1"/>
-      <c r="O554" s="156" t="s">
+      <c r="O554" s="159" t="s">
         <v>52</v>
       </c>
       <c r="P554" s="157" t="s">
@@ -31920,7 +31920,7 @@
       <c r="L555" s="1"/>
       <c r="M555" s="1"/>
       <c r="N555" s="1"/>
-      <c r="O555" s="156"/>
+      <c r="O555" s="159"/>
       <c r="P555" s="157"/>
       <c r="Q555" s="158"/>
       <c r="R555" s="3" t="s">
@@ -31942,7 +31942,7 @@
       <c r="L556" s="1"/>
       <c r="M556" s="1"/>
       <c r="N556" s="1"/>
-      <c r="O556" s="159" t="s">
+      <c r="O556" s="156" t="s">
         <v>54</v>
       </c>
       <c r="P556" s="157" t="s">
@@ -31970,7 +31970,7 @@
       <c r="L557" s="1"/>
       <c r="M557" s="1"/>
       <c r="N557" s="1"/>
-      <c r="O557" s="159"/>
+      <c r="O557" s="156"/>
       <c r="P557" s="157"/>
       <c r="Q557" s="158"/>
       <c r="R557" s="3" t="s">
@@ -31992,7 +31992,7 @@
       <c r="L558" s="1"/>
       <c r="M558" s="1"/>
       <c r="N558" s="1"/>
-      <c r="O558" s="159" t="s">
+      <c r="O558" s="156" t="s">
         <v>58</v>
       </c>
       <c r="P558" s="157" t="s">
@@ -32020,7 +32020,7 @@
       <c r="L559" s="1"/>
       <c r="M559" s="1"/>
       <c r="N559" s="1"/>
-      <c r="O559" s="159"/>
+      <c r="O559" s="156"/>
       <c r="P559" s="157"/>
       <c r="Q559" s="158"/>
       <c r="R559" s="3" t="s">
@@ -32042,7 +32042,7 @@
       <c r="L560" s="1"/>
       <c r="M560" s="1"/>
       <c r="N560" s="1"/>
-      <c r="O560" s="159" t="s">
+      <c r="O560" s="156" t="s">
         <v>62</v>
       </c>
       <c r="P560" s="157" t="s">
@@ -32070,7 +32070,7 @@
       <c r="L561" s="1"/>
       <c r="M561" s="1"/>
       <c r="N561" s="1"/>
-      <c r="O561" s="159"/>
+      <c r="O561" s="156"/>
       <c r="P561" s="157"/>
       <c r="Q561" s="158"/>
       <c r="R561" s="3" t="s">
@@ -32202,7 +32202,7 @@
       <c r="L566" s="1"/>
       <c r="M566" s="1"/>
       <c r="N566" s="1"/>
-      <c r="O566" s="156" t="s">
+      <c r="O566" s="159" t="s">
         <v>86</v>
       </c>
       <c r="P566" s="157" t="s">
@@ -32230,7 +32230,7 @@
       <c r="L567" s="1"/>
       <c r="M567" s="1"/>
       <c r="N567" s="1"/>
-      <c r="O567" s="156"/>
+      <c r="O567" s="159"/>
       <c r="P567" s="157"/>
       <c r="Q567" s="158"/>
       <c r="R567" s="3" t="s">
@@ -32252,7 +32252,7 @@
       <c r="L568" s="1"/>
       <c r="M568" s="1"/>
       <c r="N568" s="1"/>
-      <c r="O568" s="156"/>
+      <c r="O568" s="159"/>
       <c r="P568" s="157"/>
       <c r="Q568" s="158"/>
       <c r="R568" s="3" t="s">
@@ -32274,7 +32274,7 @@
       <c r="L569" s="1"/>
       <c r="M569" s="1"/>
       <c r="N569" s="1"/>
-      <c r="O569" s="156" t="s">
+      <c r="O569" s="159" t="s">
         <v>91</v>
       </c>
       <c r="P569" s="157" t="s">
@@ -32302,7 +32302,7 @@
       <c r="L570" s="1"/>
       <c r="M570" s="1"/>
       <c r="N570" s="1"/>
-      <c r="O570" s="156"/>
+      <c r="O570" s="159"/>
       <c r="P570" s="157"/>
       <c r="Q570" s="158"/>
       <c r="R570" s="3" t="s">
@@ -32324,7 +32324,7 @@
       <c r="L571" s="1"/>
       <c r="M571" s="1"/>
       <c r="N571" s="1"/>
-      <c r="O571" s="156"/>
+      <c r="O571" s="159"/>
       <c r="P571" s="157"/>
       <c r="Q571" s="158"/>
       <c r="R571" s="3" t="s">
@@ -33093,6 +33093,24 @@
   </sheetData>
   <autoFilter ref="A1:S321" xr:uid="{82619C4B-D6B1-486E-87C6-D2252668E253}"/>
   <mergeCells count="27">
+    <mergeCell ref="O544:O545"/>
+    <mergeCell ref="P544:P545"/>
+    <mergeCell ref="Q544:Q545"/>
+    <mergeCell ref="O548:O549"/>
+    <mergeCell ref="P548:P549"/>
+    <mergeCell ref="Q548:Q549"/>
+    <mergeCell ref="O558:O559"/>
+    <mergeCell ref="P558:P559"/>
+    <mergeCell ref="Q558:Q559"/>
+    <mergeCell ref="O560:O561"/>
+    <mergeCell ref="P560:P561"/>
+    <mergeCell ref="Q560:Q561"/>
+    <mergeCell ref="O566:O568"/>
+    <mergeCell ref="P566:P568"/>
+    <mergeCell ref="Q566:Q568"/>
+    <mergeCell ref="O569:O571"/>
+    <mergeCell ref="P569:P571"/>
+    <mergeCell ref="Q569:Q571"/>
     <mergeCell ref="O556:O557"/>
     <mergeCell ref="P556:P557"/>
     <mergeCell ref="Q556:Q557"/>
@@ -33102,24 +33120,6 @@
     <mergeCell ref="P554:P555"/>
     <mergeCell ref="Q554:Q555"/>
     <mergeCell ref="O550:O551"/>
-    <mergeCell ref="O566:O568"/>
-    <mergeCell ref="P566:P568"/>
-    <mergeCell ref="Q566:Q568"/>
-    <mergeCell ref="O569:O571"/>
-    <mergeCell ref="P569:P571"/>
-    <mergeCell ref="Q569:Q571"/>
-    <mergeCell ref="O558:O559"/>
-    <mergeCell ref="P558:P559"/>
-    <mergeCell ref="Q558:Q559"/>
-    <mergeCell ref="O560:O561"/>
-    <mergeCell ref="P560:P561"/>
-    <mergeCell ref="Q560:Q561"/>
-    <mergeCell ref="O544:O545"/>
-    <mergeCell ref="P544:P545"/>
-    <mergeCell ref="Q544:Q545"/>
-    <mergeCell ref="O548:O549"/>
-    <mergeCell ref="P548:P549"/>
-    <mergeCell ref="Q548:Q549"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="Q7" r:id="rId1" display="Abbreviation of the journal name. We use WoS abbreviations that can be found here: https://images.webofknowledge.com/images/help/WOS/A_abrvjt.html" xr:uid="{B4DADD6B-F846-45B3-933B-5F25CC9FEF24}"/>
@@ -39268,8 +39268,8 @@
       </c>
     </row>
     <row r="326" spans="1:7">
-      <c r="C326" s="137" t="s">
-        <v>1552</v>
+      <c r="C326" s="84" t="s">
+        <v>1630</v>
       </c>
       <c r="D326" s="154" t="s">
         <v>1653</v>
@@ -42935,7 +42935,7 @@
       <c r="A554" s="12"/>
       <c r="B554" s="12"/>
       <c r="C554" s="12"/>
-      <c r="D554" s="159" t="s">
+      <c r="D554" s="156" t="s">
         <v>35</v>
       </c>
       <c r="E554" s="157" t="s">
@@ -42952,7 +42952,7 @@
       <c r="A555" s="12"/>
       <c r="B555" s="12"/>
       <c r="C555" s="12"/>
-      <c r="D555" s="159"/>
+      <c r="D555" s="156"/>
       <c r="E555" s="157"/>
       <c r="F555" s="158"/>
       <c r="G555" s="3" t="s">
@@ -42980,7 +42980,7 @@
       <c r="A558" s="1"/>
       <c r="B558" s="1"/>
       <c r="C558" s="1"/>
-      <c r="D558" s="156" t="s">
+      <c r="D558" s="159" t="s">
         <v>42</v>
       </c>
       <c r="E558" s="157" t="s">
@@ -42997,7 +42997,7 @@
       <c r="A559" s="1"/>
       <c r="B559" s="1"/>
       <c r="C559" s="1"/>
-      <c r="D559" s="156"/>
+      <c r="D559" s="159"/>
       <c r="E559" s="157"/>
       <c r="F559" s="158"/>
       <c r="G559" s="3" t="s">
@@ -43008,7 +43008,7 @@
       <c r="A560" s="12"/>
       <c r="B560" s="12"/>
       <c r="C560" s="12"/>
-      <c r="D560" s="159" t="s">
+      <c r="D560" s="156" t="s">
         <v>45</v>
       </c>
       <c r="E560" s="157" t="s">
@@ -43025,7 +43025,7 @@
       <c r="A561" s="12"/>
       <c r="B561" s="12"/>
       <c r="C561" s="12"/>
-      <c r="D561" s="159"/>
+      <c r="D561" s="156"/>
       <c r="E561" s="157"/>
       <c r="F561" s="158"/>
       <c r="G561" s="3" t="s">
@@ -43053,7 +43053,7 @@
       <c r="A564" s="1"/>
       <c r="B564" s="1"/>
       <c r="C564" s="1"/>
-      <c r="D564" s="156" t="s">
+      <c r="D564" s="159" t="s">
         <v>52</v>
       </c>
       <c r="E564" s="157" t="s">
@@ -43070,7 +43070,7 @@
       <c r="A565" s="1"/>
       <c r="B565" s="1"/>
       <c r="C565" s="1"/>
-      <c r="D565" s="156"/>
+      <c r="D565" s="159"/>
       <c r="E565" s="157"/>
       <c r="F565" s="158"/>
       <c r="G565" s="3" t="s">
@@ -43081,7 +43081,7 @@
       <c r="A566" s="1"/>
       <c r="B566" s="1"/>
       <c r="C566" s="1"/>
-      <c r="D566" s="159" t="s">
+      <c r="D566" s="156" t="s">
         <v>54</v>
       </c>
       <c r="E566" s="157" t="s">
@@ -43098,7 +43098,7 @@
       <c r="A567" s="1"/>
       <c r="B567" s="1"/>
       <c r="C567" s="1"/>
-      <c r="D567" s="159"/>
+      <c r="D567" s="156"/>
       <c r="E567" s="157"/>
       <c r="F567" s="158"/>
       <c r="G567" s="3" t="s">
@@ -43109,7 +43109,7 @@
       <c r="A568" s="1"/>
       <c r="B568" s="1"/>
       <c r="C568" s="1"/>
-      <c r="D568" s="159" t="s">
+      <c r="D568" s="156" t="s">
         <v>58</v>
       </c>
       <c r="E568" s="157" t="s">
@@ -43126,7 +43126,7 @@
       <c r="A569" s="1"/>
       <c r="B569" s="1"/>
       <c r="C569" s="1"/>
-      <c r="D569" s="159"/>
+      <c r="D569" s="156"/>
       <c r="E569" s="157"/>
       <c r="F569" s="158"/>
       <c r="G569" s="3" t="s">
@@ -43137,7 +43137,7 @@
       <c r="A570" s="1"/>
       <c r="B570" s="1"/>
       <c r="C570" s="1"/>
-      <c r="D570" s="159" t="s">
+      <c r="D570" s="156" t="s">
         <v>62</v>
       </c>
       <c r="E570" s="157" t="s">
@@ -43154,7 +43154,7 @@
       <c r="A571" s="1"/>
       <c r="B571" s="1"/>
       <c r="C571" s="1"/>
-      <c r="D571" s="159"/>
+      <c r="D571" s="156"/>
       <c r="E571" s="157"/>
       <c r="F571" s="158"/>
       <c r="G571" s="3" t="s">
@@ -43231,7 +43231,7 @@
       <c r="A576" s="1"/>
       <c r="B576" s="1"/>
       <c r="C576" s="1"/>
-      <c r="D576" s="156" t="s">
+      <c r="D576" s="159" t="s">
         <v>86</v>
       </c>
       <c r="E576" s="157" t="s">
@@ -43248,7 +43248,7 @@
       <c r="A577" s="1"/>
       <c r="B577" s="1"/>
       <c r="C577" s="1"/>
-      <c r="D577" s="156"/>
+      <c r="D577" s="159"/>
       <c r="E577" s="157"/>
       <c r="F577" s="158"/>
       <c r="G577" s="3" t="s">
@@ -43259,7 +43259,7 @@
       <c r="A578" s="1"/>
       <c r="B578" s="1"/>
       <c r="C578" s="1"/>
-      <c r="D578" s="156"/>
+      <c r="D578" s="159"/>
       <c r="E578" s="157"/>
       <c r="F578" s="158"/>
       <c r="G578" s="3" t="s">
@@ -43270,7 +43270,7 @@
       <c r="A579" s="1"/>
       <c r="B579" s="1"/>
       <c r="C579" s="1"/>
-      <c r="D579" s="156" t="s">
+      <c r="D579" s="159" t="s">
         <v>91</v>
       </c>
       <c r="E579" s="157" t="s">
@@ -43287,7 +43287,7 @@
       <c r="A580" s="1"/>
       <c r="B580" s="1"/>
       <c r="C580" s="1"/>
-      <c r="D580" s="156"/>
+      <c r="D580" s="159"/>
       <c r="E580" s="157"/>
       <c r="F580" s="158"/>
       <c r="G580" s="3" t="s">
@@ -43298,7 +43298,7 @@
       <c r="A581" s="1"/>
       <c r="B581" s="1"/>
       <c r="C581" s="1"/>
-      <c r="D581" s="156"/>
+      <c r="D581" s="159"/>
       <c r="E581" s="157"/>
       <c r="F581" s="158"/>
       <c r="G581" s="3" t="s">
@@ -43725,24 +43725,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="D554:D555"/>
-    <mergeCell ref="E554:E555"/>
-    <mergeCell ref="F554:F555"/>
-    <mergeCell ref="D558:D559"/>
-    <mergeCell ref="E558:E559"/>
-    <mergeCell ref="F558:F559"/>
-    <mergeCell ref="D560:D561"/>
-    <mergeCell ref="E560:E561"/>
-    <mergeCell ref="F560:F561"/>
-    <mergeCell ref="D564:D565"/>
-    <mergeCell ref="E564:E565"/>
-    <mergeCell ref="F564:F565"/>
-    <mergeCell ref="D566:D567"/>
-    <mergeCell ref="E566:E567"/>
-    <mergeCell ref="F566:F567"/>
-    <mergeCell ref="D568:D569"/>
-    <mergeCell ref="E568:E569"/>
-    <mergeCell ref="F568:F569"/>
     <mergeCell ref="D579:D581"/>
     <mergeCell ref="E579:E581"/>
     <mergeCell ref="F579:F581"/>
@@ -43752,6 +43734,24 @@
     <mergeCell ref="D576:D578"/>
     <mergeCell ref="E576:E578"/>
     <mergeCell ref="F576:F578"/>
+    <mergeCell ref="D566:D567"/>
+    <mergeCell ref="E566:E567"/>
+    <mergeCell ref="F566:F567"/>
+    <mergeCell ref="D568:D569"/>
+    <mergeCell ref="E568:E569"/>
+    <mergeCell ref="F568:F569"/>
+    <mergeCell ref="D560:D561"/>
+    <mergeCell ref="E560:E561"/>
+    <mergeCell ref="F560:F561"/>
+    <mergeCell ref="D564:D565"/>
+    <mergeCell ref="E564:E565"/>
+    <mergeCell ref="F564:F565"/>
+    <mergeCell ref="D554:D555"/>
+    <mergeCell ref="E554:E555"/>
+    <mergeCell ref="F554:F555"/>
+    <mergeCell ref="D558:D559"/>
+    <mergeCell ref="E558:E559"/>
+    <mergeCell ref="F558:F559"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F7" r:id="rId1" display="Abbreviation of the journal name. We use WoS abbreviations that can be found here: https://images.webofknowledge.com/images/help/WOS/A_abrvjt.html" xr:uid="{6BB52E4D-01E2-44A6-B6CC-352383FA2940}"/>
@@ -43763,6 +43763,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4b26243c-b736-4d9c-b036-479be2ad88a1">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="432dd258-9dce-4cb3-b611-c68c0fbce7f3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005BE3C66ACF4393458051577D36AC6C25" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4e0e0d96de7fb32b1678b66c28514d8e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4b26243c-b736-4d9c-b036-479be2ad88a1" xmlns:ns3="432dd258-9dce-4cb3-b611-c68c0fbce7f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac451aab8c96dec805c937cbafca7133" ns2:_="" ns3:_="">
     <xsd:import namespace="4b26243c-b736-4d9c-b036-479be2ad88a1"/>
@@ -43963,27 +43983,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63F80AE0-5CF8-441A-8E3E-6D76A3390D5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="4b26243c-b736-4d9c-b036-479be2ad88a1"/>
+    <ds:schemaRef ds:uri="432dd258-9dce-4cb3-b611-c68c0fbce7f3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4b26243c-b736-4d9c-b036-479be2ad88a1">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="432dd258-9dce-4cb3-b611-c68c0fbce7f3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0C90B0A-DBBE-4147-B2EE-79946A8DC171}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC19592A-9F30-4B32-9428-1D9634B8A0D4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -44000,23 +44019,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0C90B0A-DBBE-4147-B2EE-79946A8DC171}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63F80AE0-5CF8-441A-8E3E-6D76A3390D5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="4b26243c-b736-4d9c-b036-479be2ad88a1"/>
-    <ds:schemaRef ds:uri="432dd258-9dce-4cb3-b611-c68c0fbce7f3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>